<commit_message>
Update inputs_outputs.xlsx & main.ipynb; replace BaseProjections and puma CSVs
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Data\Forecast\Tools\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5607A47-7EDD-4C05-85A7-A0BF6D414B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FF0E00-9DF0-4C6E-A0BB-9D6AE0295B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="12645" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>discription</t>
   </si>
@@ -62,17 +62,20 @@
     <t>kollim_factor</t>
   </si>
   <si>
-    <t>W:\Projects\בהת\263_רובע_צפון_הגבעה_הצרפתית\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>French_Hill_with_project</t>
+    <t>base_year</t>
+  </si>
+  <si>
+    <t>W:\Projects\בהת\247_שכונת_עיטם_אפרת\קבצי עבודה\תחזיות_דמוגרפיות</t>
+  </si>
+  <si>
+    <t>without_project</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -84,18 +87,6 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <charset val="177"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9CDCFE"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -118,16 +109,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -469,64 +453,69 @@
     <col min="2" max="2" width="81.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3">
-        <v>250908</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="B4">
+        <v>250427</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="B8" s="1"/>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>2040</v>
+      </c>
     </row>
     <row r="9" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
       <c r="B9" s="1"/>

</xml_diff>

<commit_message>
NS: added base year scenario feature to dev
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Data\Forecast\Tools\create_forecast_ad_hoc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FF0E00-9DF0-4C6E-A0BB-9D6AE0295B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CCDB0B7-5344-4B5A-9DAD-AD4767CC8BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -65,10 +65,10 @@
     <t>base_year</t>
   </si>
   <si>
-    <t>W:\Projects\בהת\247_שכונת_עיטם_אפרת\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>without_project</t>
+    <t>W:\Projects\בהת\262_מתחם_ביאליק_בית_שמש\קבצי עבודה\תחזיות_דמוגרפיות</t>
+  </si>
+  <si>
+    <t>bialik_with_project</t>
   </si>
 </sst>
 </file>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -447,13 +447,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" customWidth="1"/>
-    <col min="2" max="2" width="81.140625" customWidth="1"/>
+    <col min="1" max="1" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="81.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -461,7 +461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -469,7 +469,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -477,15 +477,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
-        <v>250427</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>250930</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -493,15 +493,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -509,24 +509,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8">
-        <v>2040</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NS: added 2050 files to background and added 2050 variables
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CCDB0B7-5344-4B5A-9DAD-AD4767CC8BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD54FDF-1E03-49C1-81CC-10632182B7AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3876" yWindow="2340" windowWidth="23040" windowHeight="12120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -65,10 +65,10 @@
     <t>base_year</t>
   </si>
   <si>
-    <t>W:\Projects\בהת\262_מתחם_ביאליק_בית_שמש\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>bialik_with_project</t>
+    <t>W:\Projects\בהת\מטה_בנימין_261\קבצי עבודה\תחזיות_דמוגרפיות</t>
+  </si>
+  <si>
+    <t>mate_binyamin_with_project</t>
   </si>
 </sst>
 </file>
@@ -482,7 +482,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>250930</v>
+        <v>251022</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -514,7 +514,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>2030</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
NS: created two md files in main repo. designer gudie and one script run
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD54FDF-1E03-49C1-81CC-10632182B7AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0773AF-7B1F-4153-B541-BAA5B8C39B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3876" yWindow="2340" windowWidth="23040" windowHeight="12120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -498,7 +498,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changed columns name in "if not matching files"
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0773AF-7B1F-4153-B541-BAA5B8C39B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBEF9031-437E-4D4F-BB2F-4C72AA2F21EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -65,10 +65,10 @@
     <t>base_year</t>
   </si>
   <si>
-    <t>W:\Projects\בהת\מטה_בנימין_261\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>mate_binyamin_with_project</t>
+    <t>W:\Projects\בהת\272_הדיור הממשלתי ומגרש 22 (קו צהוב)\קבצי עבודה\תחזיות_דמוגרפיות</t>
+  </si>
+  <si>
+    <t>diur_with_project</t>
   </si>
 </sst>
 </file>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -447,10 +447,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.6640625" customWidth="1"/>
-    <col min="2" max="2" width="81.109375" customWidth="1"/>
+    <col min="1" max="1" width="34.6328125" customWidth="1"/>
+    <col min="2" max="2" width="81.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -482,7 +482,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>251022</v>
+        <v>251207</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -498,7 +498,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -517,16 +517,16 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NS: fixed the code logic to be able to use the newer forecast 2020 file
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0773AF-7B1F-4153-B541-BAA5B8C39B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43DFE618-0EBF-425A-9FC3-3CCBC8204A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,10 +65,10 @@
     <t>base_year</t>
   </si>
   <si>
-    <t>W:\Projects\בהת\מטה_בנימין_261\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>mate_binyamin_with_project</t>
+    <t>W:\Projects\בהת\272_הדיור הממשלתי ומגרש 22 (קו צהוב)\קבצי עבודה\תחזיות_דמוגרפיות</t>
+  </si>
+  <si>
+    <t>diur_with_project</t>
   </si>
 </sst>
 </file>
@@ -482,7 +482,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>251022</v>
+        <v>251207</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -498,7 +498,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
AS: change paramters in ForApprovel to catch all the layer files (chnge match_basename_pattern to None)
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43DFE618-0EBF-425A-9FC3-3CCBC8204A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8AE20EC-E43F-4D08-97E3-B321CE62D70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31800" yWindow="3000" windowWidth="21600" windowHeight="12525" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -65,10 +65,10 @@
     <t>base_year</t>
   </si>
   <si>
-    <t>W:\Projects\בהת\272_הדיור הממשלתי ומגרש 22 (קו צהוב)\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>diur_with_project</t>
+    <t>W:\Projects\בהת\263_רובע_צפון_הגבעה_הצרפתית\קבצי עבודה\תחזיות_דמוגרפיות</t>
+  </si>
+  <si>
+    <t>French_Hill_with_project</t>
   </si>
 </sst>
 </file>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -447,10 +447,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.6640625" customWidth="1"/>
-    <col min="2" max="2" width="81.109375" customWidth="1"/>
+    <col min="1" max="1" width="34.6328125" customWidth="1"/>
+    <col min="2" max="2" width="81.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -482,7 +482,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>251207</v>
+        <v>250908</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -514,19 +514,19 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed slope to 5% after talk with eitan
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8AE20EC-E43F-4D08-97E3-B321CE62D70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E004625-523A-42F6-8D2D-6996E0A27647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31800" yWindow="3000" windowWidth="21600" windowHeight="12525" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-84" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -65,17 +65,17 @@
     <t>base_year</t>
   </si>
   <si>
-    <t>W:\Projects\בהת\263_רובע_צפון_הגבעה_הצרפתית\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>French_Hill_with_project</t>
+    <t>W:\Projects\תכניות מרחביות\265_בית שמש חצי מיליון\קבצי עבודה\תחזיות_דמוגרפיות</t>
+  </si>
+  <si>
+    <t>half_milion_with_project</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -86,7 +86,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -109,9 +115,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -130,7 +137,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -447,10 +454,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.6328125" customWidth="1"/>
-    <col min="2" max="2" width="81.08984375" customWidth="1"/>
+    <col min="1" max="1" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="81.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -465,7 +472,7 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -482,7 +489,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>250908</v>
+        <v>251130</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -514,19 +521,19 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>2040</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="14" x14ac:dyDescent="0.3">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:2" ht="14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:2" ht="14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:2" ht="14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
--open new feture branch+ first try hebrew for apr
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Users\Nitai\create_forecast_ad_hoc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E004625-523A-42F6-8D2D-6996E0A27647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4978D3F5-92DE-426A-9135-4057F4BDEF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-84" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1160" yWindow="600" windowWidth="21600" windowHeight="12260" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -65,10 +65,10 @@
     <t>base_year</t>
   </si>
   <si>
-    <t>W:\Projects\תכניות מרחביות\265_בית שמש חצי מיליון\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>half_milion_with_project</t>
+    <t>W:\Projects\בהת\גבעת רם - לניסוי בלבד\קבצי עבודה\תחזיות_דמוגרפיות</t>
+  </si>
+  <si>
+    <t>givaat_ram</t>
   </si>
 </sst>
 </file>
@@ -137,7 +137,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -454,10 +454,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.6640625" customWidth="1"/>
-    <col min="2" max="2" width="81.109375" customWidth="1"/>
+    <col min="1" max="1" width="34.7265625" customWidth="1"/>
+    <col min="2" max="2" width="81.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -489,7 +489,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>251130</v>
+        <v>260726</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -505,7 +505,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -521,19 +521,19 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:2" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="14" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
     </row>
   </sheetData>

</xml_diff>